<commit_message>
Add per-item amounts summing to package totals
Yellowstone line items sum to USD 61,500; operating cost line items
sum to USD 320,000. Excel totals use SUM formulas.

Co-authored-by: crios82-max <crios82-max@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/presupuesto-costo-operacion-cliente.xlsx
+++ b/docs/presupuesto-costo-operacion-cliente.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet name="PRESUPUESTO" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'PRESUPUESTO'!$A$1:$D$28</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -21,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,11 +72,6 @@
       <b val="1"/>
       <color rgb="00151A22"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="0094A3B8"/>
-      <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -130,11 +123,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2E8F0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFF5F5"/>
       </patternFill>
     </fill>
@@ -146,6 +134,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2E8F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -194,29 +187,29 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -580,21 +573,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Presupuesto - Costo de Operación</t>
+          <t>Presupuesto - Costo de Operacion</t>
         </is>
       </c>
     </row>
@@ -615,7 +608,7 @@
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Modalidad: Operación</t>
+          <t>Modalidad: Operacion</t>
         </is>
       </c>
       <c r="C6" s="5" t="n"/>
@@ -625,7 +618,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
+    <row r="8">
       <c r="B8" s="7" t="inlineStr">
         <is>
           <t>CANT.</t>
@@ -651,10 +644,8 @@
           <t>RED HUMANA</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D9" s="10" t="n">
+        <v>180000</v>
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
@@ -666,10 +657,8 @@
           <t>FE SPARTANS</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D10" s="10" t="n">
+        <v>75000</v>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
@@ -681,10 +670,8 @@
           <t>LABORATORIO BOTS</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D11" s="10" t="n">
+        <v>30000</v>
       </c>
     </row>
     <row r="12" ht="26" customHeight="1">
@@ -696,10 +683,8 @@
           <t>STAFF</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D12" s="10" t="n">
+        <v>20000</v>
       </c>
     </row>
     <row r="13" ht="26" customHeight="1">
@@ -711,21 +696,20 @@
           <t>EQUIPO GERENCIA</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="34" customHeight="1">
+      <c r="D13" s="10" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>COSTO OPERACIÓN</t>
+          <t>COSTO OPERACION</t>
         </is>
       </c>
       <c r="C15" s="5" t="n"/>
-      <c r="D15" s="12" t="n">
-        <v>320000</v>
+      <c r="D15" s="12">
+        <f>SUM(D9:D13)</f>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -740,12 +724,13 @@
     <row r="18">
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>Inversión total operación</t>
+          <t>Inversión total</t>
         </is>
       </c>
       <c r="C18" s="5" t="n"/>
-      <c r="D18" s="16" t="n">
-        <v>320000</v>
+      <c r="D18" s="16">
+        <f>D15</f>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -758,9 +743,9 @@
     <row r="21">
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>• Estructura operativa: Red Humana, FE Spartans, Laboratorio Bots, Staff y Equipo de Gerencia.
+          <t>• Cada concepto incluye su monto; el total es la suma de los ítems.
 • Validez del presupuesto: 15 días. Montos en dólares estadounidenses (USD).
-• Costo de operación: USD 320,000.</t>
+• Total: USD 320,000.</t>
         </is>
       </c>
       <c r="C21" s="19" t="n"/>
@@ -779,7 +764,7 @@
     <row r="25">
       <c r="B25" s="20" t="inlineStr">
         <is>
-          <t>COSTO OPERACIÓN · Presupuesto cliente · 1 hoja</t>
+          <t>COSTO OPERACION · Presupuesto cliente · 1 hoja</t>
         </is>
       </c>
     </row>
@@ -795,6 +780,5 @@
     <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update operating cost budget quantities and uneven amounts
Set Red Humana 9,012, Espartanos 515, Cuentas 3,500 and Staff 15,
use non-round line totals ending nonzero, and render totals in black.

Co-authored-by: crios82-max <crios82-max@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/presupuesto-costo-operacion-cliente.xlsx
+++ b/docs/presupuesto-costo-operacion-cliente.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,19 +76,25 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00111111"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="00111A2D"/>
       <sz val="13"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00C41E3A"/>
+      <color rgb="00111111"/>
       <sz val="16"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00C41E3A"/>
+      <color rgb="00111111"/>
       <sz val="14"/>
     </font>
     <font>
@@ -104,7 +110,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -123,7 +129,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF5F5"/>
+        <fgColor rgb="00E2E8F0"/>
       </patternFill>
     </fill>
     <fill>
@@ -134,11 +140,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2E8F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -187,13 +188,13 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -201,15 +202,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -575,19 +576,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D25"/>
+  <dimension ref="B2:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Presupuesto - Costo de Operacion</t>
+          <t>Presupuesto - Costo de Operación</t>
         </is>
       </c>
     </row>
@@ -601,14 +602,14 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Red Humana, FE Spartans, Laboratorio Bots, Staff y Equipo de Gerencia</t>
+          <t>Red Humana, Espartanos, Cuentas y Staff</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Modalidad: Operacion</t>
+          <t>Modalidad: Operación</t>
         </is>
       </c>
       <c r="C6" s="5" t="n"/>
@@ -637,7 +638,7 @@
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="B9" s="8" t="n">
-        <v>9000</v>
+        <v>9012</v>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
@@ -645,38 +646,38 @@
         </is>
       </c>
       <c r="D9" s="10" t="n">
-        <v>180000</v>
+        <v>179483</v>
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="B10" s="8" t="n">
-        <v>500</v>
+        <v>515</v>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>FE SPARTANS</t>
+          <t>ESPARTANOS</t>
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>75000</v>
+        <v>74857</v>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
       <c r="B11" s="8" t="n">
-        <v>20</v>
+        <v>3500</v>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>LABORATORIO BOTS</t>
+          <t>CUENTAS</t>
         </is>
       </c>
       <c r="D11" s="10" t="n">
-        <v>30000</v>
+        <v>47629</v>
       </c>
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="B12" s="8" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
@@ -684,70 +685,60 @@
         </is>
       </c>
       <c r="D12" s="10" t="n">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="13" ht="26" customHeight="1">
-      <c r="B13" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>EQUIPO GERENCIA</t>
-        </is>
-      </c>
-      <c r="D13" s="10" t="n">
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>COSTO OPERACION</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="12">
-        <f>SUM(D9:D13)</f>
-        <v/>
-      </c>
+        <v>18547</v>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>COSTO OPERACIÓN</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="12" t="n">
+        <v>320516</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>RESUMEN</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="14" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>RESUMEN</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="14" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="15" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>Inversión total</t>
         </is>
       </c>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="16">
-        <f>D15</f>
-        <v/>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="16" t="n">
+        <v>320516</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>Condiciones</t>
+        </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="17" t="inlineStr">
-        <is>
-          <t>Condiciones</t>
-        </is>
-      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>• Cada concepto tiene su monto; el total es la suma de las líneas.
+• Validez del presupuesto: 15 días. Montos en dólares estadounidenses (USD).
+• Costo de operación: USD 320,516.</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="19" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>• Cada concepto incluye su monto; el total es la suma de los ítems.
-• Validez del presupuesto: 15 días. Montos en dólares estadounidenses (USD).
-• Total: USD 320,000.</t>
-        </is>
-      </c>
+      <c r="B21" s="19" t="n"/>
       <c r="C21" s="19" t="n"/>
       <c r="D21" s="19" t="n"/>
     </row>
@@ -756,15 +747,10 @@
       <c r="C22" s="19" t="n"/>
       <c r="D22" s="19" t="n"/>
     </row>
-    <row r="23">
-      <c r="B23" s="19" t="n"/>
-      <c r="C23" s="19" t="n"/>
-      <c r="D23" s="19" t="n"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="20" t="inlineStr">
-        <is>
-          <t>COSTO OPERACION · Presupuesto cliente · 1 hoja</t>
+    <row r="24">
+      <c r="B24" s="20" t="inlineStr">
+        <is>
+          <t>COSTO OPERACIÓN · Presupuesto cliente · 1 hoja</t>
         </is>
       </c>
     </row>
@@ -772,11 +758,11 @@
   <mergeCells count="8">
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B15:C15"/>
     <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B21:D23"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B20:D22"/>
+    <mergeCell ref="B17:C17"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>